<commit_message>
fix: universe vs comps count
</commit_message>
<xml_diff>
--- a/ddfda77d-a4ea-4731-b5ab-3929032f42ff.xlsx
+++ b/ddfda77d-a4ea-4731-b5ab-3929032f42ff.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6667fcbc27a88bd9/Pancho Main/Cursor/Fran-Facu Proyecto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97C6BF87-9D5E-4D93-A255-7D6033CD414A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7252FA5-307F-4194-A523-1DA1F9B4ED9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="69">
   <si>
     <t>PARÁMETROS DEL DEAL</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>Net Inc ($mm)</t>
+  </si>
+  <si>
+    <t>Gross ($mm)</t>
   </si>
   <si>
     <t>Deuda ($mm)</t>
@@ -422,9 +425,9 @@
     <xf numFmtId="3" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -727,7 +730,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:V17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -738,18 +741,18 @@
     <col min="6" max="6" width="60" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
     <col min="8" max="9" width="14" customWidth="1"/>
-    <col min="10" max="11" width="13" customWidth="1"/>
-    <col min="12" max="12" width="15" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="9" customWidth="1"/>
-    <col min="15" max="17" width="13" customWidth="1"/>
-    <col min="18" max="18" width="12" customWidth="1"/>
-    <col min="19" max="21" width="13" customWidth="1"/>
+    <col min="10" max="12" width="13" customWidth="1"/>
+    <col min="13" max="13" width="15" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="9" customWidth="1"/>
+    <col min="16" max="18" width="13" customWidth="1"/>
+    <col min="19" max="19" width="12" customWidth="1"/>
+    <col min="20" max="22" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
-        <v>63</v>
+    <row r="1" spans="1:22" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
+        <v>64</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -771,10 +774,11 @@
       <c r="S1" s="25"/>
       <c r="T1" s="25"/>
       <c r="U1" s="25"/>
-    </row>
-    <row r="2" spans="1:21" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
-        <v>64</v>
+      <c r="V1" s="25"/>
+    </row>
+    <row r="2" spans="1:22" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="26" t="s">
+        <v>65</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -796,9 +800,10 @@
       <c r="S2" s="25"/>
       <c r="T2" s="25"/>
       <c r="U2" s="25"/>
-    </row>
-    <row r="3" spans="1:21" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="V2" s="25"/>
+    </row>
+    <row r="3" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -862,25 +867,28 @@
       <c r="U4" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="V4" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G5" s="4">
         <v>716924</v>
@@ -892,60 +900,63 @@
         <v>77670</v>
       </c>
       <c r="J5" s="4">
+        <v>360510</v>
+      </c>
+      <c r="K5" s="4">
         <v>178547</v>
       </c>
-      <c r="K5" s="4">
+      <c r="L5" s="4">
         <v>123029</v>
       </c>
-      <c r="L5" s="4">
-        <v>2281492.7000000002</v>
-      </c>
       <c r="M5" s="4">
+        <v>2257017.1</v>
+      </c>
+      <c r="N5" s="4">
         <v>2260148.7000000002</v>
       </c>
-      <c r="N5" s="5">
-        <v>29.6</v>
-      </c>
-      <c r="O5" s="6">
+      <c r="O5" s="5">
+        <v>29.3</v>
+      </c>
+      <c r="P5" s="6">
         <v>13.6</v>
       </c>
-      <c r="P5" s="7">
+      <c r="Q5" s="7">
         <v>1576000</v>
       </c>
-      <c r="Q5" s="6">
+      <c r="R5" s="6">
         <v>23.1</v>
       </c>
-      <c r="R5" s="6">
+      <c r="S5" s="6">
         <v>10.8</v>
       </c>
-      <c r="S5" s="6">
+      <c r="T5" s="6">
         <v>50.3</v>
       </c>
-      <c r="T5" s="5">
+      <c r="U5" s="5">
         <v>3.2</v>
       </c>
-      <c r="U5" s="5">
+      <c r="V5" s="5">
         <v>13.7</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G6" s="10">
         <v>34534</v>
@@ -957,60 +968,63 @@
         <v>208</v>
       </c>
       <c r="J6" s="10">
+        <v>10141</v>
+      </c>
+      <c r="K6" s="10">
         <v>4635</v>
       </c>
-      <c r="K6" s="10">
+      <c r="L6" s="10">
         <v>6318</v>
       </c>
-      <c r="L6" s="10">
-        <v>35732</v>
-      </c>
       <c r="M6" s="10">
+        <v>35320.699999999997</v>
+      </c>
+      <c r="N6" s="10">
         <v>32741.8</v>
       </c>
-      <c r="N6" s="11">
-        <v>177.7</v>
-      </c>
-      <c r="O6" s="12">
+      <c r="O6" s="11">
+        <v>175.6</v>
+      </c>
+      <c r="P6" s="12">
         <v>10.9</v>
       </c>
-      <c r="P6" s="13">
+      <c r="Q6" s="13">
         <v>108000</v>
       </c>
-      <c r="Q6" s="12">
+      <c r="R6" s="12">
         <v>3.5</v>
       </c>
-      <c r="R6" s="12">
+      <c r="S6" s="12">
         <v>0.6</v>
       </c>
-      <c r="S6" s="12">
+      <c r="T6" s="12">
         <v>29.4</v>
       </c>
-      <c r="T6" s="11">
+      <c r="U6" s="11">
         <v>0.9</v>
       </c>
-      <c r="U6" s="11">
+      <c r="V6" s="11">
         <v>27.3</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G7" s="4">
         <v>13717</v>
@@ -1022,60 +1036,63 @@
         <v>935</v>
       </c>
       <c r="J7" s="4">
+        <v>7109</v>
+      </c>
+      <c r="K7" s="4">
         <v>3290</v>
       </c>
-      <c r="K7" s="4">
+      <c r="L7" s="4">
         <v>5506</v>
       </c>
-      <c r="L7" s="4">
-        <v>71350.2</v>
-      </c>
       <c r="M7" s="4">
+        <v>69499.5</v>
+      </c>
+      <c r="N7" s="4">
         <v>65845.5</v>
       </c>
-      <c r="N7" s="5">
-        <v>77.099999999999994</v>
-      </c>
-      <c r="O7" s="6">
+      <c r="O7" s="5">
+        <v>75.099999999999994</v>
+      </c>
+      <c r="P7" s="6">
         <v>37.700000000000003</v>
       </c>
-      <c r="P7" s="7">
+      <c r="Q7" s="7">
         <v>31400</v>
       </c>
-      <c r="Q7" s="6">
+      <c r="R7" s="6">
         <v>10.7</v>
       </c>
-      <c r="R7" s="6">
+      <c r="S7" s="6">
         <v>6.8</v>
       </c>
-      <c r="S7" s="6">
+      <c r="T7" s="6">
         <v>51.8</v>
       </c>
-      <c r="T7" s="5">
+      <c r="U7" s="5">
         <v>4.8</v>
       </c>
-      <c r="U7" s="5">
+      <c r="V7" s="5">
         <v>44.7</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G8" s="10">
         <v>12584.2</v>
@@ -1087,60 +1104,63 @@
         <v>206.4</v>
       </c>
       <c r="J8" s="10">
+        <v>3720.2</v>
+      </c>
+      <c r="K8" s="10">
         <v>558.9</v>
       </c>
-      <c r="K8" s="10">
+      <c r="L8" s="10">
         <v>701.5</v>
       </c>
-      <c r="L8" s="10">
-        <v>9906</v>
-      </c>
       <c r="M8" s="10">
+        <v>9794</v>
+      </c>
+      <c r="N8" s="10">
         <v>9555.9</v>
       </c>
-      <c r="N8" s="11">
-        <v>48.7</v>
-      </c>
-      <c r="O8" s="12">
+      <c r="O8" s="11">
+        <v>48.2</v>
+      </c>
+      <c r="P8" s="12">
         <v>8.3000000000000007</v>
       </c>
-      <c r="P8" s="13">
+      <c r="Q8" s="13">
         <v>18000</v>
       </c>
-      <c r="Q8" s="12">
+      <c r="R8" s="12">
         <v>2.8</v>
       </c>
-      <c r="R8" s="12">
+      <c r="S8" s="12">
         <v>1.6</v>
       </c>
-      <c r="S8" s="12">
+      <c r="T8" s="12">
         <v>29.6</v>
       </c>
-      <c r="T8" s="11">
+      <c r="U8" s="11">
         <v>0.8</v>
       </c>
-      <c r="U8" s="11">
+      <c r="V8" s="11">
         <v>27.5</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G9" s="4">
         <v>11100</v>
@@ -1152,60 +1172,63 @@
         <v>1996</v>
       </c>
       <c r="J9" s="4">
+        <v>7931</v>
+      </c>
+      <c r="K9" s="4">
         <v>7182</v>
       </c>
-      <c r="K9" s="4">
+      <c r="L9" s="4">
         <v>2919</v>
       </c>
-      <c r="L9" s="4">
-        <v>40912.800000000003</v>
-      </c>
       <c r="M9" s="4">
+        <v>40612.199999999997</v>
+      </c>
+      <c r="N9" s="4">
         <v>44126</v>
       </c>
-      <c r="N9" s="5">
-        <v>21.2</v>
-      </c>
-      <c r="O9" s="6">
+      <c r="O9" s="5">
+        <v>21.1</v>
+      </c>
+      <c r="P9" s="6">
         <v>15</v>
       </c>
-      <c r="P9" s="7">
+      <c r="Q9" s="7">
         <v>12300</v>
       </c>
-      <c r="Q9" s="6">
+      <c r="R9" s="6">
         <v>26.7</v>
       </c>
-      <c r="R9" s="6">
+      <c r="S9" s="6">
         <v>18</v>
       </c>
-      <c r="S9" s="6">
+      <c r="T9" s="6">
         <v>71.5</v>
       </c>
-      <c r="T9" s="5">
+      <c r="U9" s="5">
         <v>4</v>
       </c>
-      <c r="U9" s="5">
+      <c r="V9" s="5">
         <v>14.9</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G10" s="10">
         <v>3742</v>
@@ -1217,60 +1240,63 @@
         <v>438</v>
       </c>
       <c r="J10" s="10">
+        <v>2758</v>
+      </c>
+      <c r="K10" s="10">
         <v>36</v>
       </c>
-      <c r="K10" s="10">
+      <c r="L10" s="10">
         <v>687</v>
       </c>
-      <c r="L10" s="10">
-        <v>9902.7000000000007</v>
-      </c>
       <c r="M10" s="10">
+        <v>10007.799999999999</v>
+      </c>
+      <c r="N10" s="10">
         <v>8430.9</v>
       </c>
-      <c r="N10" s="11">
-        <v>23.6</v>
-      </c>
-      <c r="O10" s="12">
+      <c r="O10" s="11">
+        <v>23.8</v>
+      </c>
+      <c r="P10" s="12">
         <v>12.3</v>
       </c>
-      <c r="P10" s="13">
+      <c r="Q10" s="13">
         <v>3600</v>
       </c>
-      <c r="Q10" s="12">
+      <c r="R10" s="12">
         <v>16</v>
       </c>
-      <c r="R10" s="12">
+      <c r="S10" s="12">
         <v>11.7</v>
       </c>
-      <c r="S10" s="12">
+      <c r="T10" s="12">
         <v>73.7</v>
       </c>
-      <c r="T10" s="11">
+      <c r="U10" s="11">
         <v>2.2999999999999998</v>
       </c>
-      <c r="U10" s="11">
+      <c r="V10" s="11">
         <v>14.1</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G11" s="4">
         <v>2883.5</v>
@@ -1282,60 +1308,63 @@
         <v>163</v>
       </c>
       <c r="J11" s="4">
+        <v>2065.6999999999998</v>
+      </c>
+      <c r="K11" s="4">
         <v>3115.1</v>
       </c>
-      <c r="K11" s="4">
+      <c r="L11" s="4">
         <v>1619.9</v>
       </c>
-      <c r="L11" s="4">
-        <v>5291.6</v>
-      </c>
       <c r="M11" s="4">
+        <v>5184</v>
+      </c>
+      <c r="N11" s="4">
         <v>6580.9</v>
       </c>
-      <c r="N11" s="5">
-        <v>38.6</v>
-      </c>
-      <c r="O11" s="6">
+      <c r="O11" s="5">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="P11" s="6">
         <v>3.5</v>
       </c>
-      <c r="P11" s="7">
+      <c r="Q11" s="7">
         <v>2375</v>
       </c>
-      <c r="Q11" s="6">
+      <c r="R11" s="6">
         <v>16.5</v>
       </c>
-      <c r="R11" s="6">
+      <c r="S11" s="6">
         <v>5.7</v>
       </c>
-      <c r="S11" s="6">
+      <c r="T11" s="6">
         <v>71.599999999999994</v>
       </c>
-      <c r="T11" s="5">
+      <c r="U11" s="5">
         <v>2.2999999999999998</v>
       </c>
-      <c r="U11" s="5">
+      <c r="V11" s="5">
         <v>13.8</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G12" s="10">
         <v>1225.7</v>
@@ -1347,60 +1376,63 @@
         <v>61.7</v>
       </c>
       <c r="J12" s="10">
+        <v>655.8</v>
+      </c>
+      <c r="K12" s="10">
         <v>32.5</v>
       </c>
-      <c r="K12" s="10">
+      <c r="L12" s="10">
         <v>292.3</v>
       </c>
-      <c r="L12" s="10">
-        <v>1620.7</v>
-      </c>
       <c r="M12" s="10">
+        <v>1584.3</v>
+      </c>
+      <c r="N12" s="10">
         <v>1319.5</v>
       </c>
-      <c r="N12" s="11">
-        <v>26.4</v>
-      </c>
-      <c r="O12" s="12">
+      <c r="O12" s="11">
+        <v>25.8</v>
+      </c>
+      <c r="P12" s="12">
         <v>10.4</v>
       </c>
-      <c r="P12" s="13">
+      <c r="Q12" s="13">
         <v>1664</v>
       </c>
-      <c r="Q12" s="12">
+      <c r="R12" s="12">
         <v>6.6</v>
       </c>
-      <c r="R12" s="12">
+      <c r="S12" s="12">
         <v>5</v>
       </c>
-      <c r="S12" s="12">
+      <c r="T12" s="12">
         <v>53.5</v>
       </c>
-      <c r="T12" s="11">
+      <c r="U12" s="11">
         <v>1.1000000000000001</v>
       </c>
-      <c r="U12" s="11">
+      <c r="V12" s="11">
         <v>16.399999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G13" s="4">
         <v>888.5</v>
@@ -1412,58 +1444,61 @@
         <v>68.3</v>
       </c>
       <c r="J13" s="4">
+        <v>436.2</v>
+      </c>
+      <c r="K13" s="4">
         <v>23.5</v>
       </c>
-      <c r="K13" s="4">
+      <c r="L13" s="4">
         <v>622.79999999999995</v>
       </c>
-      <c r="L13" s="4">
-        <v>5532.2</v>
-      </c>
       <c r="M13" s="4">
+        <v>5472</v>
+      </c>
+      <c r="N13" s="4">
         <v>4903.1000000000004</v>
       </c>
-      <c r="N13" s="5">
-        <v>83.6</v>
-      </c>
-      <c r="O13" s="6">
+      <c r="O13" s="5">
+        <v>82.7</v>
+      </c>
+      <c r="P13" s="6">
         <v>28</v>
       </c>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="6">
+      <c r="Q13" s="7"/>
+      <c r="R13" s="6">
         <v>24.7</v>
       </c>
-      <c r="R13" s="6">
+      <c r="S13" s="6">
         <v>7.7</v>
       </c>
-      <c r="S13" s="6">
+      <c r="T13" s="6">
         <v>49.1</v>
       </c>
-      <c r="T13" s="5">
+      <c r="U13" s="5">
         <v>5.5</v>
       </c>
-      <c r="U13" s="5">
+      <c r="V13" s="5">
         <v>22.3</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G14" s="10">
         <v>475.6</v>
@@ -1475,45 +1510,48 @@
         <v>29.8</v>
       </c>
       <c r="J14" s="10">
+        <v>215.7</v>
+      </c>
+      <c r="K14" s="10">
         <v>13.8</v>
       </c>
-      <c r="K14" s="10">
+      <c r="L14" s="10">
         <v>181.4</v>
       </c>
-      <c r="L14" s="10">
-        <v>927.9</v>
-      </c>
       <c r="M14" s="10">
+        <v>928.6</v>
+      </c>
+      <c r="N14" s="10">
         <v>720.6</v>
       </c>
-      <c r="N14" s="11">
+      <c r="O14" s="11">
         <v>32.5</v>
       </c>
-      <c r="O14" s="12">
+      <c r="P14" s="12">
         <v>-0.9</v>
       </c>
-      <c r="P14" s="13">
+      <c r="Q14" s="13">
         <v>818</v>
       </c>
-      <c r="Q14" s="12">
+      <c r="R14" s="12">
         <v>10.1</v>
       </c>
-      <c r="R14" s="12">
+      <c r="S14" s="12">
         <v>6.3</v>
       </c>
-      <c r="S14" s="12">
+      <c r="T14" s="12">
         <v>45.4</v>
       </c>
-      <c r="T14" s="11">
+      <c r="U14" s="11">
         <v>1.5</v>
       </c>
-      <c r="U14" s="11">
+      <c r="V14" s="11">
         <v>15.1</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G16" s="15">
         <f>MEDIAN(G5:G14)</f>
@@ -1527,46 +1565,46 @@
         <f>MEDIAN(I5:I14)</f>
         <v>207.2</v>
       </c>
-      <c r="L16" s="15">
-        <f>MEDIAN(L5:L14)</f>
-        <v>9904.35</v>
-      </c>
       <c r="M16" s="15">
         <f>MEDIAN(M5:M14)</f>
+        <v>9900.9</v>
+      </c>
+      <c r="N16" s="15">
+        <f>MEDIAN(N5:N14)</f>
         <v>8993.4</v>
       </c>
-      <c r="N16" s="16">
-        <f>MEDIAN(N5:N14)</f>
-        <v>35.549999999999997</v>
-      </c>
-      <c r="O16" s="17">
+      <c r="O16" s="16">
         <f>MEDIAN(O5:O14)</f>
+        <v>35.15</v>
+      </c>
+      <c r="P16" s="17">
+        <f>MEDIAN(P5:P14)</f>
         <v>11.600000000000001</v>
-      </c>
-      <c r="Q16" s="17">
-        <f>MEDIAN(Q5:Q14)</f>
-        <v>13.35</v>
       </c>
       <c r="R16" s="17">
         <f>MEDIAN(R5:R14)</f>
-        <v>6.55</v>
+        <v>13.35</v>
       </c>
       <c r="S16" s="17">
         <f>MEDIAN(S5:S14)</f>
+        <v>6.55</v>
+      </c>
+      <c r="T16" s="17">
+        <f>MEDIAN(T5:T14)</f>
         <v>51.05</v>
-      </c>
-      <c r="T16" s="16">
-        <f>MEDIAN(T5:T14)</f>
-        <v>2.2999999999999998</v>
       </c>
       <c r="U16" s="16">
         <f>MEDIAN(U5:U14)</f>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="V16" s="16">
+        <f>MEDIAN(V5:V14)</f>
         <v>15.75</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G17" s="15">
         <f>AVERAGE(G5:G14)</f>
@@ -1580,47 +1618,47 @@
         <f>AVERAGE(I5:I14)</f>
         <v>8177.62</v>
       </c>
-      <c r="L17" s="15">
-        <f>AVERAGE(L5:L14)</f>
-        <v>246266.88000000006</v>
-      </c>
       <c r="M17" s="15">
         <f>AVERAGE(M5:M14)</f>
+        <v>243542.02000000002</v>
+      </c>
+      <c r="N17" s="15">
+        <f>AVERAGE(N5:N14)</f>
         <v>243437.28999999998</v>
       </c>
-      <c r="N17" s="16">
-        <f>AVERAGE(N5:N14)</f>
-        <v>55.9</v>
-      </c>
-      <c r="O17" s="17">
+      <c r="O17" s="16">
         <f>AVERAGE(O5:O14)</f>
+        <v>55.190000000000012</v>
+      </c>
+      <c r="P17" s="17">
+        <f>AVERAGE(P5:P14)</f>
         <v>13.879999999999999</v>
-      </c>
-      <c r="Q17" s="17">
-        <f>AVERAGE(Q5:Q14)</f>
-        <v>14.069999999999999</v>
       </c>
       <c r="R17" s="17">
         <f>AVERAGE(R5:R14)</f>
-        <v>7.42</v>
+        <v>14.069999999999999</v>
       </c>
       <c r="S17" s="17">
         <f>AVERAGE(S5:S14)</f>
+        <v>7.42</v>
+      </c>
+      <c r="T17" s="17">
+        <f>AVERAGE(T5:T14)</f>
         <v>52.589999999999996</v>
-      </c>
-      <c r="T17" s="16">
-        <f>AVERAGE(T5:T14)</f>
-        <v>2.64</v>
       </c>
       <c r="U17" s="16">
         <f>AVERAGE(U5:U14)</f>
+        <v>2.64</v>
+      </c>
+      <c r="V17" s="16">
+        <f>AVERAGE(V5:V14)</f>
         <v>20.98</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:U1"/>
-    <mergeCell ref="A2:U2"/>
+    <mergeCell ref="A2:V2"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1628,7 +1666,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:U26"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -1639,21 +1677,21 @@
     <col min="6" max="6" width="60" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
     <col min="8" max="9" width="14" customWidth="1"/>
-    <col min="10" max="11" width="13" customWidth="1"/>
-    <col min="12" max="12" width="15" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="9" customWidth="1"/>
-    <col min="15" max="17" width="13" customWidth="1"/>
-    <col min="18" max="18" width="12" customWidth="1"/>
-    <col min="19" max="21" width="13" customWidth="1"/>
+    <col min="10" max="12" width="13" customWidth="1"/>
+    <col min="13" max="13" width="15" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="9" customWidth="1"/>
+    <col min="16" max="18" width="13" customWidth="1"/>
+    <col min="19" max="19" width="12" customWidth="1"/>
+    <col min="20" max="22" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
@@ -1661,7 +1699,7 @@
         <v>28893</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
         <v>2</v>
       </c>
@@ -1669,7 +1707,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
         <v>3</v>
       </c>
@@ -1677,9 +1715,9 @@
         <v>300</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="26" t="s">
+    <row r="5" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:22" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="24" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="25"/>
@@ -1702,9 +1740,10 @@
       <c r="S6" s="25"/>
       <c r="T6" s="25"/>
       <c r="U6" s="25"/>
-    </row>
-    <row r="7" spans="1:21" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
+      <c r="V6" s="25"/>
+    </row>
+    <row r="7" spans="1:22" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="25"/>
@@ -1727,8 +1766,9 @@
       <c r="S7" s="25"/>
       <c r="T7" s="25"/>
       <c r="U7" s="25"/>
-    </row>
-    <row r="8" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="V7" s="25"/>
+    </row>
+    <row r="8" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1792,25 +1832,28 @@
       <c r="U8" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="9" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="V8" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G9" s="4">
         <v>716924</v>
@@ -1822,60 +1865,63 @@
         <v>77670</v>
       </c>
       <c r="J9" s="4">
+        <v>360510</v>
+      </c>
+      <c r="K9" s="4">
         <v>178547</v>
       </c>
-      <c r="K9" s="4">
+      <c r="L9" s="4">
         <v>123029</v>
       </c>
-      <c r="L9" s="4">
-        <v>2281492.7000000002</v>
-      </c>
       <c r="M9" s="4">
+        <v>2257017.1</v>
+      </c>
+      <c r="N9" s="4">
         <v>2260148.7000000002</v>
       </c>
-      <c r="N9" s="5">
-        <v>29.6</v>
-      </c>
-      <c r="O9" s="6">
+      <c r="O9" s="5">
+        <v>29.3</v>
+      </c>
+      <c r="P9" s="6">
         <v>13.6</v>
       </c>
-      <c r="P9" s="7">
+      <c r="Q9" s="7">
         <v>1576000</v>
       </c>
-      <c r="Q9" s="6">
+      <c r="R9" s="6">
         <v>23.1</v>
       </c>
-      <c r="R9" s="6">
+      <c r="S9" s="6">
         <v>10.8</v>
       </c>
-      <c r="S9" s="6">
+      <c r="T9" s="6">
         <v>50.3</v>
       </c>
-      <c r="T9" s="5">
+      <c r="U9" s="5">
         <v>3.2</v>
       </c>
-      <c r="U9" s="5">
+      <c r="V9" s="5">
         <v>13.7</v>
       </c>
     </row>
-    <row r="10" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G10" s="10">
         <v>34534</v>
@@ -1887,60 +1933,63 @@
         <v>208</v>
       </c>
       <c r="J10" s="10">
+        <v>10141</v>
+      </c>
+      <c r="K10" s="10">
         <v>4635</v>
       </c>
-      <c r="K10" s="10">
+      <c r="L10" s="10">
         <v>6318</v>
       </c>
-      <c r="L10" s="10">
-        <v>35732</v>
-      </c>
       <c r="M10" s="10">
+        <v>35320.699999999997</v>
+      </c>
+      <c r="N10" s="10">
         <v>32741.8</v>
       </c>
-      <c r="N10" s="11">
-        <v>177.7</v>
-      </c>
-      <c r="O10" s="12">
+      <c r="O10" s="11">
+        <v>175.6</v>
+      </c>
+      <c r="P10" s="12">
         <v>10.9</v>
       </c>
-      <c r="P10" s="13">
+      <c r="Q10" s="13">
         <v>108000</v>
       </c>
-      <c r="Q10" s="12">
+      <c r="R10" s="12">
         <v>3.5</v>
       </c>
-      <c r="R10" s="12">
+      <c r="S10" s="12">
         <v>0.6</v>
       </c>
-      <c r="S10" s="12">
+      <c r="T10" s="12">
         <v>29.4</v>
       </c>
-      <c r="T10" s="11">
+      <c r="U10" s="11">
         <v>0.9</v>
       </c>
-      <c r="U10" s="11">
+      <c r="V10" s="11">
         <v>27.3</v>
       </c>
     </row>
-    <row r="11" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G11" s="4">
         <v>13717</v>
@@ -1952,60 +2001,63 @@
         <v>935</v>
       </c>
       <c r="J11" s="4">
+        <v>7109</v>
+      </c>
+      <c r="K11" s="4">
         <v>3290</v>
       </c>
-      <c r="K11" s="4">
+      <c r="L11" s="4">
         <v>5506</v>
       </c>
-      <c r="L11" s="4">
-        <v>71350.2</v>
-      </c>
       <c r="M11" s="4">
+        <v>69499.5</v>
+      </c>
+      <c r="N11" s="4">
         <v>65845.5</v>
       </c>
-      <c r="N11" s="5">
-        <v>77.099999999999994</v>
-      </c>
-      <c r="O11" s="6">
+      <c r="O11" s="5">
+        <v>75.099999999999994</v>
+      </c>
+      <c r="P11" s="6">
         <v>37.700000000000003</v>
       </c>
-      <c r="P11" s="7">
+      <c r="Q11" s="7">
         <v>31400</v>
       </c>
-      <c r="Q11" s="6">
+      <c r="R11" s="6">
         <v>10.7</v>
       </c>
-      <c r="R11" s="6">
+      <c r="S11" s="6">
         <v>6.8</v>
       </c>
-      <c r="S11" s="6">
+      <c r="T11" s="6">
         <v>51.8</v>
       </c>
-      <c r="T11" s="5">
+      <c r="U11" s="5">
         <v>4.8</v>
       </c>
-      <c r="U11" s="5">
+      <c r="V11" s="5">
         <v>44.7</v>
       </c>
     </row>
-    <row r="12" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G12" s="10">
         <v>12584.2</v>
@@ -2017,60 +2069,63 @@
         <v>206.4</v>
       </c>
       <c r="J12" s="10">
+        <v>3720.2</v>
+      </c>
+      <c r="K12" s="10">
         <v>558.9</v>
       </c>
-      <c r="K12" s="10">
+      <c r="L12" s="10">
         <v>701.5</v>
       </c>
-      <c r="L12" s="10">
-        <v>9906</v>
-      </c>
       <c r="M12" s="10">
+        <v>9794</v>
+      </c>
+      <c r="N12" s="10">
         <v>9555.9</v>
       </c>
-      <c r="N12" s="11">
-        <v>48.7</v>
-      </c>
-      <c r="O12" s="12">
+      <c r="O12" s="11">
+        <v>48.2</v>
+      </c>
+      <c r="P12" s="12">
         <v>8.3000000000000007</v>
       </c>
-      <c r="P12" s="13">
+      <c r="Q12" s="13">
         <v>18000</v>
       </c>
-      <c r="Q12" s="12">
+      <c r="R12" s="12">
         <v>2.8</v>
       </c>
-      <c r="R12" s="12">
+      <c r="S12" s="12">
         <v>1.6</v>
       </c>
-      <c r="S12" s="12">
+      <c r="T12" s="12">
         <v>29.6</v>
       </c>
-      <c r="T12" s="11">
+      <c r="U12" s="11">
         <v>0.8</v>
       </c>
-      <c r="U12" s="11">
+      <c r="V12" s="11">
         <v>27.5</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G13" s="4">
         <v>11100</v>
@@ -2082,60 +2137,63 @@
         <v>1996</v>
       </c>
       <c r="J13" s="4">
+        <v>7931</v>
+      </c>
+      <c r="K13" s="4">
         <v>7182</v>
       </c>
-      <c r="K13" s="4">
+      <c r="L13" s="4">
         <v>2919</v>
       </c>
-      <c r="L13" s="4">
-        <v>40912.800000000003</v>
-      </c>
       <c r="M13" s="4">
+        <v>40612.199999999997</v>
+      </c>
+      <c r="N13" s="4">
         <v>44126</v>
       </c>
-      <c r="N13" s="5">
-        <v>21.2</v>
-      </c>
-      <c r="O13" s="6">
+      <c r="O13" s="5">
+        <v>21.1</v>
+      </c>
+      <c r="P13" s="6">
         <v>15</v>
       </c>
-      <c r="P13" s="7">
+      <c r="Q13" s="7">
         <v>12300</v>
       </c>
-      <c r="Q13" s="6">
+      <c r="R13" s="6">
         <v>26.7</v>
       </c>
-      <c r="R13" s="6">
+      <c r="S13" s="6">
         <v>18</v>
       </c>
-      <c r="S13" s="6">
+      <c r="T13" s="6">
         <v>71.5</v>
       </c>
-      <c r="T13" s="5">
+      <c r="U13" s="5">
         <v>4</v>
       </c>
-      <c r="U13" s="5">
+      <c r="V13" s="5">
         <v>14.9</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G14" s="10">
         <v>3742</v>
@@ -2147,60 +2205,63 @@
         <v>438</v>
       </c>
       <c r="J14" s="10">
+        <v>2758</v>
+      </c>
+      <c r="K14" s="10">
         <v>36</v>
       </c>
-      <c r="K14" s="10">
+      <c r="L14" s="10">
         <v>687</v>
       </c>
-      <c r="L14" s="10">
-        <v>9902.7000000000007</v>
-      </c>
       <c r="M14" s="10">
+        <v>10007.799999999999</v>
+      </c>
+      <c r="N14" s="10">
         <v>8430.9</v>
       </c>
-      <c r="N14" s="11">
-        <v>23.6</v>
-      </c>
-      <c r="O14" s="12">
+      <c r="O14" s="11">
+        <v>23.8</v>
+      </c>
+      <c r="P14" s="12">
         <v>12.3</v>
       </c>
-      <c r="P14" s="13">
+      <c r="Q14" s="13">
         <v>3600</v>
       </c>
-      <c r="Q14" s="12">
+      <c r="R14" s="12">
         <v>16</v>
       </c>
-      <c r="R14" s="12">
+      <c r="S14" s="12">
         <v>11.7</v>
       </c>
-      <c r="S14" s="12">
+      <c r="T14" s="12">
         <v>73.7</v>
       </c>
-      <c r="T14" s="11">
+      <c r="U14" s="11">
         <v>2.2999999999999998</v>
       </c>
-      <c r="U14" s="11">
+      <c r="V14" s="11">
         <v>14.1</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G15" s="4">
         <v>2883.5</v>
@@ -2212,60 +2273,63 @@
         <v>163</v>
       </c>
       <c r="J15" s="4">
+        <v>2065.6999999999998</v>
+      </c>
+      <c r="K15" s="4">
         <v>3115.1</v>
       </c>
-      <c r="K15" s="4">
+      <c r="L15" s="4">
         <v>1619.9</v>
       </c>
-      <c r="L15" s="4">
-        <v>5291.6</v>
-      </c>
       <c r="M15" s="4">
+        <v>5184</v>
+      </c>
+      <c r="N15" s="4">
         <v>6580.9</v>
       </c>
-      <c r="N15" s="5">
-        <v>38.6</v>
-      </c>
-      <c r="O15" s="6">
+      <c r="O15" s="5">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="P15" s="6">
         <v>3.5</v>
       </c>
-      <c r="P15" s="7">
+      <c r="Q15" s="7">
         <v>2375</v>
       </c>
-      <c r="Q15" s="6">
+      <c r="R15" s="6">
         <v>16.5</v>
       </c>
-      <c r="R15" s="6">
+      <c r="S15" s="6">
         <v>5.7</v>
       </c>
-      <c r="S15" s="6">
+      <c r="T15" s="6">
         <v>71.599999999999994</v>
       </c>
-      <c r="T15" s="5">
+      <c r="U15" s="5">
         <v>2.2999999999999998</v>
       </c>
-      <c r="U15" s="5">
+      <c r="V15" s="5">
         <v>13.8</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G16" s="10">
         <v>1225.7</v>
@@ -2277,60 +2341,63 @@
         <v>61.7</v>
       </c>
       <c r="J16" s="10">
+        <v>655.8</v>
+      </c>
+      <c r="K16" s="10">
         <v>32.5</v>
       </c>
-      <c r="K16" s="10">
+      <c r="L16" s="10">
         <v>292.3</v>
       </c>
-      <c r="L16" s="10">
-        <v>1620.7</v>
-      </c>
       <c r="M16" s="10">
+        <v>1584.3</v>
+      </c>
+      <c r="N16" s="10">
         <v>1319.5</v>
       </c>
-      <c r="N16" s="11">
-        <v>26.4</v>
-      </c>
-      <c r="O16" s="12">
+      <c r="O16" s="11">
+        <v>25.8</v>
+      </c>
+      <c r="P16" s="12">
         <v>10.4</v>
       </c>
-      <c r="P16" s="13">
+      <c r="Q16" s="13">
         <v>1664</v>
       </c>
-      <c r="Q16" s="12">
+      <c r="R16" s="12">
         <v>6.6</v>
       </c>
-      <c r="R16" s="12">
+      <c r="S16" s="12">
         <v>5</v>
       </c>
-      <c r="S16" s="12">
+      <c r="T16" s="12">
         <v>53.5</v>
       </c>
-      <c r="T16" s="11">
+      <c r="U16" s="11">
         <v>1.1000000000000001</v>
       </c>
-      <c r="U16" s="11">
+      <c r="V16" s="11">
         <v>16.399999999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G17" s="4">
         <v>888.5</v>
@@ -2342,43 +2409,46 @@
         <v>68.3</v>
       </c>
       <c r="J17" s="4">
+        <v>436.2</v>
+      </c>
+      <c r="K17" s="4">
         <v>23.5</v>
       </c>
-      <c r="K17" s="4">
+      <c r="L17" s="4">
         <v>622.79999999999995</v>
       </c>
-      <c r="L17" s="4">
-        <v>5532.2</v>
-      </c>
       <c r="M17" s="4">
+        <v>5472</v>
+      </c>
+      <c r="N17" s="4">
         <v>4903.1000000000004</v>
       </c>
-      <c r="N17" s="5">
-        <v>83.6</v>
-      </c>
-      <c r="O17" s="6">
+      <c r="O17" s="5">
+        <v>82.7</v>
+      </c>
+      <c r="P17" s="6">
         <v>28</v>
       </c>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="6">
+      <c r="Q17" s="7"/>
+      <c r="R17" s="6">
         <v>24.7</v>
       </c>
-      <c r="R17" s="6">
+      <c r="S17" s="6">
         <v>7.7</v>
       </c>
-      <c r="S17" s="6">
+      <c r="T17" s="6">
         <v>49.1</v>
       </c>
-      <c r="T17" s="5">
+      <c r="U17" s="5">
         <v>5.5</v>
       </c>
-      <c r="U17" s="5">
+      <c r="V17" s="5">
         <v>22.3</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G19" s="15">
         <f>MEDIAN(G9:G17)</f>
@@ -2392,46 +2462,46 @@
         <f>MEDIAN(I9:I17)</f>
         <v>208</v>
       </c>
-      <c r="L19" s="15">
-        <f>MEDIAN(L9:L17)</f>
-        <v>9906</v>
-      </c>
       <c r="M19" s="15">
         <f>MEDIAN(M9:M17)</f>
+        <v>10007.799999999999</v>
+      </c>
+      <c r="N19" s="15">
+        <f>MEDIAN(N9:N17)</f>
         <v>9555.9</v>
       </c>
-      <c r="N19" s="16">
-        <f>MEDIAN(N9:N17)</f>
-        <v>38.6</v>
-      </c>
-      <c r="O19" s="17">
+      <c r="O19" s="16">
         <f>MEDIAN(O9:O17)</f>
+        <v>37.799999999999997</v>
+      </c>
+      <c r="P19" s="17">
+        <f>MEDIAN(P9:P17)</f>
         <v>12.3</v>
-      </c>
-      <c r="Q19" s="17">
-        <f>MEDIAN(Q9:Q17)</f>
-        <v>16</v>
       </c>
       <c r="R19" s="17">
         <f>MEDIAN(R9:R17)</f>
-        <v>6.8</v>
+        <v>16</v>
       </c>
       <c r="S19" s="17">
         <f>MEDIAN(S9:S17)</f>
+        <v>6.8</v>
+      </c>
+      <c r="T19" s="17">
+        <f>MEDIAN(T9:T17)</f>
         <v>51.8</v>
-      </c>
-      <c r="T19" s="16">
-        <f>MEDIAN(T9:T17)</f>
-        <v>2.2999999999999998</v>
       </c>
       <c r="U19" s="16">
         <f>MEDIAN(U9:U17)</f>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="V19" s="16">
+        <f>MEDIAN(V9:V17)</f>
         <v>16.399999999999999</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G20" s="15">
         <f>AVERAGE(G9:G17)</f>
@@ -2445,49 +2515,49 @@
         <f>AVERAGE(I9:I17)</f>
         <v>9082.9333333333325</v>
       </c>
-      <c r="L20" s="15">
-        <f>AVERAGE(L9:L17)</f>
-        <v>273526.76666666678</v>
-      </c>
       <c r="M20" s="15">
         <f>AVERAGE(M9:M17)</f>
+        <v>270499.06666666665</v>
+      </c>
+      <c r="N20" s="15">
+        <f>AVERAGE(N9:N17)</f>
         <v>270405.81111111108</v>
       </c>
-      <c r="N20" s="16">
-        <f>AVERAGE(N9:N17)</f>
-        <v>58.5</v>
-      </c>
-      <c r="O20" s="17">
+      <c r="O20" s="16">
         <f>AVERAGE(O9:O17)</f>
+        <v>57.711111111111123</v>
+      </c>
+      <c r="P20" s="17">
+        <f>AVERAGE(P9:P17)</f>
         <v>15.52222222222222</v>
-      </c>
-      <c r="Q20" s="17">
-        <f>AVERAGE(Q9:Q17)</f>
-        <v>14.511111111111111</v>
       </c>
       <c r="R20" s="17">
         <f>AVERAGE(R9:R17)</f>
-        <v>7.5444444444444452</v>
+        <v>14.511111111111111</v>
       </c>
       <c r="S20" s="17">
         <f>AVERAGE(S9:S17)</f>
+        <v>7.5444444444444452</v>
+      </c>
+      <c r="T20" s="17">
+        <f>AVERAGE(T9:T17)</f>
         <v>53.388888888888886</v>
-      </c>
-      <c r="T20" s="16">
-        <f>AVERAGE(T9:T17)</f>
-        <v>2.7666666666666671</v>
       </c>
       <c r="U20" s="16">
         <f>AVERAGE(U9:U17)</f>
+        <v>2.7666666666666671</v>
+      </c>
+      <c r="V20" s="16">
+        <f>AVERAGE(V9:V17)</f>
         <v>21.633333333333336</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A24" s="19" t="s">
         <v>1</v>
       </c>
@@ -2496,28 +2566,28 @@
         <v>28893</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A25" s="19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B25" s="23">
-        <f>$B$2*T19</f>
+        <f>$B$2*U19</f>
         <v>66453.899999999994</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26" s="19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B26" s="23">
-        <f>$B$2*(Q19/100)*U19</f>
+        <f>$B$2*(R19/100)*V19</f>
         <v>75815.231999999989</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A7:U7"/>
-    <mergeCell ref="A6:U6"/>
+    <mergeCell ref="A6:V6"/>
+    <mergeCell ref="A7:V7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>